<commit_message>
Movilización: February 2025 confirmed as campaign month (operational problem in January)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BsMRKE8hArHddZxwmwcNWn
</commit_message>
<xml_diff>
--- a/movilizacion/entregables/Auditoria_Evaluacion_SierraCol_v5.xlsx
+++ b/movilizacion/entregables/Auditoria_Evaluacion_SierraCol_v5.xlsx
@@ -1322,25 +1322,25 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Febrero tiene 1 movilización (13-feb, INFA4562 a 12 km, 60 h) y paga el cargo fijo de 1 movilización: 133.751 (PS) y 181.054 (EC). ¿La campaña arrancó en febrero o fue un movimiento suelto?</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>Media</t>
+          <t>Febrero tiene 1 movilización y paga el cargo fijo de 1 movilización: 133.751 (PS) y 181.054 (EC). CONFIRMADO por SierraCol: el pozo de enero tuvo problemas operativos y duró casi un mes; febrero sí fue mes de campaña. El cálculo es correcto y muestra el riesgo real: un pozo complicado deja un mes con pocas movilizaciones y el tercerizado cobra el cargo fijo igual.</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Baja</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>133751</v>
+        <v>0</v>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Indeterminado</t>
+          <t>Neutro (correcto)</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Confirmar el inicio de la campaña; si no era campaña, ese cargo no aplica.</t>
+          <t>Sin corrección. Usarlo como ejemplo del riesgo de meses con baja frecuencia.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Movilización: Work Order tariffs are a cap (confirmed); outsourced has no cap — reframed across simulator, audit and deck
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BsMRKE8hArHddZxwmwcNWn
</commit_message>
<xml_diff>
--- a/movilizacion/entregables/Auditoria_Evaluacion_SierraCol_v5.xlsx
+++ b/movilizacion/entregables/Auditoria_Evaluacion_SierraCol_v5.xlsx
@@ -565,7 +565,7 @@
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>• Sesgo: de 17 hallazgos, 9 favorecen al tercerizado y solo 1 al WO (el bono del WO por mover más rápido, que no está en ningún lado); el resto son neutros o indeterminados. Es un sesgo sistemático, igual que en la evaluación previa.</t>
+          <t>• Sesgo: de 17 hallazgos, 10 favorecen al tercerizado y ninguno al WO (incluido el tope del WO: se compara contra el WO más caro posible); el resto son neutros o indeterminados. Es un sesgo sistemático, igual que en la evaluación previa.</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Bono del Work Order por mover más rápido no está considerado: las tarifas WO son los ítems 'más de X horas' (banda más lenta). Si el contratista movió más rápido, el WO real fue más caro.</t>
+          <t>CONFIRMADO por SierraCol: las tarifas WO son el tope (lo máximo, con movilización rápida); si tarda más se paga una tarifa fija menor. Ambas evaluaciones comparan contra el WO más caro posible, y el tercerizado no tiene tope. En 2025 las movilizaciones lentas habrían pagado menos en el WO.</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -1297,12 +1297,12 @@
       <c r="G15" s="7" t="n"/>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Favorece WO</t>
+          <t>Favorece tercerizado</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Pedir la tabla del WO por bandas de horas y aplicarla con las horas reales.</t>
+          <t>Dejar el WO en su tope como cota superior y declararlo: el ahorro calculado es el máximo posible frente al WO.</t>
         </is>
       </c>
     </row>
@@ -2035,22 +2035,22 @@
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Bono del WO por mover más rápido</t>
+          <t>Tope del WO (tarifa máxima, con piso si tarda más)</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No explícito</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Parámetro (pendiente tabla)</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Favorecería al tercerizado.</t>
+          <t>El WO está acotado; el tercerizado no.</t>
         </is>
       </c>
     </row>

</xml_diff>